<commit_message>
Modificaciones en cuadro economico 2
</commit_message>
<xml_diff>
--- a/data/datos_clientes.xlsx
+++ b/data/datos_clientes.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6c51ee1e6bfdc4f0/1. Voltia/Cosas Nico/Reporte_Fotovoltaico/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="8_{FA7FC9A3-D387-CA45-9740-697372029857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75D3C5D4-A6D7-314D-8A50-6BBB55547492}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="8_{FA7FC9A3-D387-CA45-9740-697372029857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13B8A4D2-9006-6E41-8F8C-421F07AFA8A2}"/>
   <bookViews>
-    <workbookView xWindow="17120" yWindow="680" windowWidth="17080" windowHeight="20000" xr2:uid="{ED5A8133-1C70-5642-9072-1075FB072BB4}"/>
+    <workbookView xWindow="-5760" yWindow="1200" windowWidth="17080" windowHeight="19860" xr2:uid="{ED5A8133-1C70-5642-9072-1075FB072BB4}"/>
   </bookViews>
   <sheets>
-    <sheet name="datos" sheetId="1" r:id="rId1"/>
+    <sheet name="constantes" sheetId="2" r:id="rId1"/>
+    <sheet name="datos" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
   <si>
     <t>cliente</t>
   </si>
@@ -75,6 +76,21 @@
   </si>
   <si>
     <t>Ruben Penedo</t>
+  </si>
+  <si>
+    <t>inversion</t>
+  </si>
+  <si>
+    <t>fecha_inst</t>
+  </si>
+  <si>
+    <t>2025-05</t>
+  </si>
+  <si>
+    <t>2024-06</t>
+  </si>
+  <si>
+    <t>ahorro_promesa</t>
   </si>
 </sst>
 </file>
@@ -137,10 +153,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -459,22 +471,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B8AB1E5-2594-104C-BB21-8CE123B04319}">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F4">
+        <v>7500</v>
+      </c>
+      <c r="G4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F5">
+        <v>8000</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C386E9ED-A108-6D41-A270-797EE8E6AE81}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,28 +599,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -511,28 +616,19 @@
         <v>9</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>757</v>
       </c>
       <c r="D4">
-        <v>757</v>
+        <v>276</v>
       </c>
       <c r="E4">
-        <v>276</v>
-      </c>
-      <c r="F4">
         <v>620</v>
       </c>
-      <c r="G4" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="H4" s="1">
-        <v>0.75</v>
-      </c>
-      <c r="I4" s="1">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -540,28 +636,19 @@
         <v>9</v>
       </c>
       <c r="C5">
-        <v>8</v>
+        <v>1234</v>
       </c>
       <c r="D5">
-        <v>1234</v>
+        <v>628</v>
       </c>
       <c r="E5">
-        <v>628</v>
-      </c>
-      <c r="F5">
         <v>967</v>
       </c>
-      <c r="G5" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="H5" s="1">
-        <v>0.75</v>
-      </c>
-      <c r="I5" s="1">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -569,28 +656,19 @@
         <v>10</v>
       </c>
       <c r="C6">
-        <v>9</v>
+        <v>636</v>
       </c>
       <c r="D6">
-        <v>636</v>
+        <v>261</v>
       </c>
       <c r="E6">
-        <v>261</v>
-      </c>
-      <c r="F6">
         <v>516</v>
       </c>
-      <c r="G6" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="H6" s="1">
-        <v>0.75</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -598,26 +676,17 @@
         <v>10</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>1002</v>
       </c>
       <c r="D7">
-        <v>1002</v>
+        <v>529</v>
       </c>
       <c r="E7">
-        <v>529</v>
-      </c>
-      <c r="F7">
         <v>806</v>
       </c>
-      <c r="G7" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="H7" s="1">
-        <v>0.75</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0.1</v>
-      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Primera version funcional en html
</commit_message>
<xml_diff>
--- a/data/datos_clientes.xlsx
+++ b/data/datos_clientes.xlsx
@@ -2,21 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6c51ee1e6bfdc4f0/1. Voltia/Cosas Nico/Reporte_Fotovoltaico/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="8_{FA7FC9A3-D387-CA45-9740-697372029857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13B8A4D2-9006-6E41-8F8C-421F07AFA8A2}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="8_{FA7FC9A3-D387-CA45-9740-697372029857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50E27F6B-B12A-486F-BE3B-59D0CFD684CF}"/>
   <bookViews>
-    <workbookView xWindow="-5760" yWindow="1200" windowWidth="17080" windowHeight="19860" xr2:uid="{ED5A8133-1C70-5642-9072-1075FB072BB4}"/>
+    <workbookView xWindow="820" yWindow="680" windowWidth="17080" windowHeight="19860" activeTab="2" xr2:uid="{ED5A8133-1C70-5642-9072-1075FB072BB4}"/>
   </bookViews>
   <sheets>
     <sheet name="constantes" sheetId="2" r:id="rId1"/>
-    <sheet name="datos" sheetId="1" r:id="rId2"/>
+    <sheet name="constantes_globales" sheetId="3" r:id="rId2"/>
+    <sheet name="datos" sheetId="1" r:id="rId3"/>
+    <sheet name="Hoja3" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,11 +39,50 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="35">
   <si>
     <t>cliente</t>
   </si>
   <si>
+    <t>potencia_contratada_kw</t>
+  </si>
+  <si>
+    <t>pct_punta</t>
+  </si>
+  <si>
+    <t>pct_llano</t>
+  </si>
+  <si>
+    <t>pct_valle</t>
+  </si>
+  <si>
+    <t>inversion</t>
+  </si>
+  <si>
+    <t>fecha_inst</t>
+  </si>
+  <si>
+    <t>ahorro_promesa</t>
+  </si>
+  <si>
+    <t>pot_inst</t>
+  </si>
+  <si>
+    <t>Rodrigo Alvarez</t>
+  </si>
+  <si>
+    <t>2024-08</t>
+  </si>
+  <si>
+    <t>Ruben Penedo</t>
+  </si>
+  <si>
+    <t>2025-05</t>
+  </si>
+  <si>
+    <t>Dólar</t>
+  </si>
+  <si>
     <t>mes</t>
   </si>
   <si>
@@ -54,43 +95,55 @@
     <t>exportacion_kwh</t>
   </si>
   <si>
-    <t>potencia_contratada_kw</t>
-  </si>
-  <si>
-    <t>pct_punta</t>
-  </si>
-  <si>
-    <t>pct_llano</t>
-  </si>
-  <si>
-    <t>pct_valle</t>
+    <t>2024-09</t>
+  </si>
+  <si>
+    <t>2024-10</t>
+  </si>
+  <si>
+    <t>2024-11</t>
+  </si>
+  <si>
+    <t>2024-12</t>
+  </si>
+  <si>
+    <t>2025-01</t>
+  </si>
+  <si>
+    <t>2025-02</t>
+  </si>
+  <si>
+    <t>2025-03</t>
+  </si>
+  <si>
+    <t>2025-04</t>
+  </si>
+  <si>
+    <t>2025-06</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
   </si>
   <si>
     <t>2026-01</t>
   </si>
   <si>
     <t>2026-02</t>
-  </si>
-  <si>
-    <t>Rodrigo Alvarez</t>
-  </si>
-  <si>
-    <t>Ruben Penedo</t>
-  </si>
-  <si>
-    <t>inversion</t>
-  </si>
-  <si>
-    <t>fecha_inst</t>
-  </si>
-  <si>
-    <t>2025-05</t>
-  </si>
-  <si>
-    <t>2024-06</t>
-  </si>
-  <si>
-    <t>ahorro_promesa</t>
   </si>
 </sst>
 </file>
@@ -153,6 +206,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -472,8 +529,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B8AB1E5-2594-104C-BB21-8CE123B04319}">
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5" bestFit="1" customWidth="1"/>
@@ -483,35 +540,38 @@
     <col min="7" max="7" width="9.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>9</v>
@@ -526,18 +586,21 @@
         <v>0.1</v>
       </c>
       <c r="F4">
-        <v>7500</v>
+        <v>7039</v>
       </c>
       <c r="G4" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="H4">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>4510</v>
+      </c>
+      <c r="I4">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>8</v>
@@ -555,18 +618,21 @@
         <v>8000</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H5">
         <v>6000</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -577,9 +643,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FD86A25-3D5E-9F4B-8DB6-7DFD268C5B51}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C386E9ED-A108-6D41-A270-797EE8E6AE81}">
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -596,33 +680,73 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
-      </c>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2">
+        <v>518</v>
+      </c>
+      <c r="D2">
+        <v>576</v>
+      </c>
+      <c r="E2">
+        <v>341</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3">
+        <v>628</v>
+      </c>
+      <c r="D3">
+        <v>494</v>
+      </c>
+      <c r="E3">
+        <v>443</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="C4">
-        <v>757</v>
+        <v>696</v>
       </c>
       <c r="D4">
-        <v>276</v>
+        <v>453</v>
       </c>
       <c r="E4">
-        <v>620</v>
+        <v>522</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -630,19 +754,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C5">
-        <v>1234</v>
+        <v>750</v>
       </c>
       <c r="D5">
-        <v>628</v>
+        <v>479</v>
       </c>
       <c r="E5">
-        <v>967</v>
+        <v>543</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -650,43 +774,336 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C6">
-        <v>636</v>
+        <v>776</v>
       </c>
       <c r="D6">
-        <v>261</v>
+        <v>451</v>
       </c>
       <c r="E6">
-        <v>516</v>
-      </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
+        <v>581</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7">
+        <v>564</v>
+      </c>
+      <c r="D7">
+        <v>417</v>
+      </c>
+      <c r="E7">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>509</v>
+      </c>
+      <c r="D8">
+        <v>515</v>
+      </c>
+      <c r="E8">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9">
+        <v>435</v>
+      </c>
+      <c r="D9">
+        <v>528</v>
+      </c>
+      <c r="E9">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7">
+      <c r="C10">
+        <v>325</v>
+      </c>
+      <c r="D10">
+        <v>559</v>
+      </c>
+      <c r="E10">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11">
+        <v>289</v>
+      </c>
+      <c r="D11">
+        <v>626</v>
+      </c>
+      <c r="E11">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>293</v>
+      </c>
+      <c r="D12">
+        <v>523</v>
+      </c>
+      <c r="E12">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13">
+        <v>392</v>
+      </c>
+      <c r="D13">
+        <v>360</v>
+      </c>
+      <c r="E13">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14">
+        <v>471</v>
+      </c>
+      <c r="D14">
+        <v>318</v>
+      </c>
+      <c r="E14">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15">
+        <v>625</v>
+      </c>
+      <c r="D15">
+        <v>299</v>
+      </c>
+      <c r="E15">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16">
+        <v>707</v>
+      </c>
+      <c r="D16">
+        <v>266</v>
+      </c>
+      <c r="E16">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17">
+        <v>750</v>
+      </c>
+      <c r="D17">
+        <v>312</v>
+      </c>
+      <c r="E17">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18">
+        <v>757</v>
+      </c>
+      <c r="D18">
+        <v>276</v>
+      </c>
+      <c r="E18">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19">
+        <v>636</v>
+      </c>
+      <c r="D19">
+        <v>260</v>
+      </c>
+      <c r="E19">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20">
+        <v>1234</v>
+      </c>
+      <c r="D20">
+        <v>628</v>
+      </c>
+      <c r="E20">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21">
         <v>1002</v>
       </c>
-      <c r="D7">
+      <c r="D21">
         <v>529</v>
       </c>
-      <c r="E7">
+      <c r="E21">
         <v>806</v>
       </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E372C8EC-44EC-D249-B34B-B908D14C2850}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1">
+        <v>1234</v>
+      </c>
+      <c r="D1">
+        <v>628</v>
+      </c>
+      <c r="E1">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2">
+        <v>636</v>
+      </c>
+      <c r="D2">
+        <v>261</v>
+      </c>
+      <c r="E2">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3">
+        <v>1002</v>
+      </c>
+      <c r="D3">
+        <v>529</v>
+      </c>
+      <c r="E3">
+        <v>806</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
previo a testing por clientes
</commit_message>
<xml_diff>
--- a/data/datos_clientes.xlsx
+++ b/data/datos_clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6c51ee1e6bfdc4f0/1. Voltia/Cosas Nico/Reporte_Fotovoltaico/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="8_{FA7FC9A3-D387-CA45-9740-697372029857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50E27F6B-B12A-486F-BE3B-59D0CFD684CF}"/>
+  <xr:revisionPtr revIDLastSave="325" documentId="8_{FA7FC9A3-D387-CA45-9740-697372029857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6939CC41-365C-7F4E-A989-11487CF51298}"/>
   <bookViews>
     <workbookView xWindow="820" yWindow="680" windowWidth="17080" windowHeight="19860" activeTab="2" xr2:uid="{ED5A8133-1C70-5642-9072-1075FB072BB4}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="constantes" sheetId="2" r:id="rId1"/>
     <sheet name="constantes_globales" sheetId="3" r:id="rId2"/>
     <sheet name="datos" sheetId="1" r:id="rId3"/>
-    <sheet name="Hoja3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="39">
   <si>
     <t>cliente</t>
   </si>
@@ -77,48 +76,54 @@
     <t>Ruben Penedo</t>
   </si>
   <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>David Raij</t>
+  </si>
+  <si>
+    <t>2024-12</t>
+  </si>
+  <si>
+    <t>Dólar</t>
+  </si>
+  <si>
+    <t>mes</t>
+  </si>
+  <si>
+    <t>generacion_kwh</t>
+  </si>
+  <si>
+    <t>consumo_kwh</t>
+  </si>
+  <si>
+    <t>exportacion_kwh</t>
+  </si>
+  <si>
+    <t>2024-09</t>
+  </si>
+  <si>
+    <t>2024-10</t>
+  </si>
+  <si>
+    <t>2024-11</t>
+  </si>
+  <si>
+    <t>2025-01</t>
+  </si>
+  <si>
+    <t>2025-02</t>
+  </si>
+  <si>
+    <t>2025-03</t>
+  </si>
+  <si>
+    <t>2025-04</t>
+  </si>
+  <si>
     <t>2025-05</t>
   </si>
   <si>
-    <t>Dólar</t>
-  </si>
-  <si>
-    <t>mes</t>
-  </si>
-  <si>
-    <t>generacion_kwh</t>
-  </si>
-  <si>
-    <t>consumo_kwh</t>
-  </si>
-  <si>
-    <t>exportacion_kwh</t>
-  </si>
-  <si>
-    <t>2024-09</t>
-  </si>
-  <si>
-    <t>2024-10</t>
-  </si>
-  <si>
-    <t>2024-11</t>
-  </si>
-  <si>
-    <t>2024-12</t>
-  </si>
-  <si>
-    <t>2025-01</t>
-  </si>
-  <si>
-    <t>2025-02</t>
-  </si>
-  <si>
-    <t>2025-03</t>
-  </si>
-  <si>
-    <t>2025-04</t>
-  </si>
-  <si>
     <t>2025-06</t>
   </si>
   <si>
@@ -128,9 +133,6 @@
     <t>2025-08</t>
   </si>
   <si>
-    <t>2025-09</t>
-  </si>
-  <si>
     <t>2025-10</t>
   </si>
   <si>
@@ -144,6 +146,15 @@
   </si>
   <si>
     <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fernando </t>
+  </si>
+  <si>
+    <t>Fernando</t>
   </si>
 </sst>
 </file>
@@ -206,10 +217,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -615,27 +622,75 @@
         <v>0.1</v>
       </c>
       <c r="F5">
-        <v>8000</v>
+        <v>7026</v>
       </c>
       <c r="G5" t="s">
         <v>12</v>
       </c>
       <c r="H5">
-        <v>6000</v>
+        <v>6400</v>
       </c>
       <c r="I5">
-        <v>8</v>
+        <v>7.74</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F6">
+        <v>7442</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6">
+        <v>4200</v>
+      </c>
+      <c r="I6">
+        <v>4.25</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F7">
+        <v>7442</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7">
+        <v>4200</v>
+      </c>
+      <c r="I7">
+        <v>4.25</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -649,7 +704,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1">
         <v>40</v>
@@ -662,7 +717,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C386E9ED-A108-6D41-A270-797EE8E6AE81}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
@@ -680,16 +735,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -697,7 +752,7 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2">
         <v>518</v>
@@ -717,7 +772,7 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C3">
         <v>628</v>
@@ -737,7 +792,7 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C4">
         <v>696</v>
@@ -757,7 +812,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C5">
         <v>750</v>
@@ -777,7 +832,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6">
         <v>776</v>
@@ -794,7 +849,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7">
         <v>564</v>
@@ -811,7 +866,7 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8">
         <v>509</v>
@@ -828,7 +883,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9">
         <v>435</v>
@@ -845,7 +900,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C10">
         <v>325</v>
@@ -862,7 +917,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C11">
         <v>289</v>
@@ -879,7 +934,7 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C12">
         <v>293</v>
@@ -896,7 +951,7 @@
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C13">
         <v>392</v>
@@ -913,7 +968,7 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="C14">
         <v>471</v>
@@ -930,7 +985,7 @@
         <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C15">
         <v>625</v>
@@ -947,7 +1002,7 @@
         <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16">
         <v>707</v>
@@ -964,7 +1019,7 @@
         <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C17">
         <v>750</v>
@@ -981,7 +1036,7 @@
         <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C18">
         <v>757</v>
@@ -998,7 +1053,7 @@
         <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C19">
         <v>636</v>
@@ -1015,16 +1070,16 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C20">
-        <v>1234</v>
+        <v>846</v>
       </c>
       <c r="D20">
-        <v>628</v>
+        <v>545</v>
       </c>
       <c r="E20">
-        <v>967</v>
+        <v>648</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1032,77 +1087,645 @@
         <v>11</v>
       </c>
       <c r="B21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21">
+        <v>1158</v>
+      </c>
+      <c r="D21">
+        <v>540</v>
+      </c>
+      <c r="E21">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22">
+        <v>1235</v>
+      </c>
+      <c r="D22">
+        <v>649</v>
+      </c>
+      <c r="E22">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" t="s">
         <v>34</v>
       </c>
-      <c r="C21">
+      <c r="C23">
+        <v>1234</v>
+      </c>
+      <c r="D23">
+        <v>628</v>
+      </c>
+      <c r="E23">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24">
         <v>1002</v>
       </c>
-      <c r="D21">
+      <c r="D24">
         <v>529</v>
       </c>
-      <c r="E21">
+      <c r="E24">
         <v>806</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E372C8EC-44EC-D249-B34B-B908D14C2850}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25">
+        <v>767</v>
+      </c>
+      <c r="D25">
+        <v>888</v>
+      </c>
+      <c r="E25">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26">
+        <v>422</v>
+      </c>
+      <c r="D26">
+        <v>543</v>
+      </c>
+      <c r="E26">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27">
+        <v>881</v>
+      </c>
+      <c r="D27">
+        <v>531</v>
+      </c>
+      <c r="E27">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28">
+        <v>645</v>
+      </c>
+      <c r="D28">
+        <v>588</v>
+      </c>
+      <c r="E28">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29">
+        <v>617</v>
+      </c>
+      <c r="D29">
+        <v>513</v>
+      </c>
+      <c r="E29">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30">
+        <v>492</v>
+      </c>
+      <c r="D30">
+        <v>477</v>
+      </c>
+      <c r="E30">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31">
+        <v>324</v>
+      </c>
+      <c r="D31">
+        <v>566</v>
+      </c>
+      <c r="E31">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>13</v>
+      </c>
+      <c r="B32" t="s">
+        <v>28</v>
+      </c>
+      <c r="C32">
+        <v>300</v>
+      </c>
+      <c r="D32">
+        <v>616</v>
+      </c>
+      <c r="E32">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" t="s">
+        <v>29</v>
+      </c>
+      <c r="C33">
+        <v>297</v>
+      </c>
+      <c r="D33">
+        <v>606</v>
+      </c>
+      <c r="E33">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34">
+        <v>396</v>
+      </c>
+      <c r="D34">
+        <v>609</v>
+      </c>
+      <c r="E34">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35">
+        <v>600</v>
+      </c>
+      <c r="D35">
+        <v>563</v>
+      </c>
+      <c r="E35">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36">
+        <v>745</v>
+      </c>
+      <c r="D36">
+        <v>539</v>
+      </c>
+      <c r="E36">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37">
+        <v>787</v>
+      </c>
+      <c r="D37">
+        <v>490</v>
+      </c>
+      <c r="E37">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" t="s">
         <v>33</v>
       </c>
-      <c r="C1">
-        <v>1234</v>
-      </c>
-      <c r="D1">
-        <v>628</v>
-      </c>
-      <c r="E1">
-        <v>967</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C38">
+        <v>818</v>
+      </c>
+      <c r="D38">
+        <v>680</v>
+      </c>
+      <c r="E38">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" t="s">
         <v>34</v>
       </c>
-      <c r="C2">
-        <v>636</v>
-      </c>
-      <c r="D2">
-        <v>261</v>
-      </c>
-      <c r="E2">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C39">
+        <v>855</v>
+      </c>
+      <c r="D39">
+        <v>557</v>
+      </c>
+      <c r="E39">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40">
+        <v>755</v>
+      </c>
+      <c r="D40">
+        <v>468</v>
+      </c>
+      <c r="E40">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41">
+        <v>664</v>
+      </c>
+      <c r="D41">
+        <v>470</v>
+      </c>
+      <c r="E41">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" t="s">
+        <v>36</v>
+      </c>
+      <c r="C42">
+        <v>522</v>
+      </c>
+      <c r="D42">
+        <v>573</v>
+      </c>
+      <c r="E42">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>38</v>
+      </c>
+      <c r="B43" t="s">
+        <v>35</v>
+      </c>
+      <c r="C43">
+        <v>755</v>
+      </c>
+      <c r="D43">
+        <v>468</v>
+      </c>
+      <c r="E43">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>38</v>
+      </c>
+      <c r="B44" t="s">
+        <v>36</v>
+      </c>
+      <c r="C44">
+        <v>664</v>
+      </c>
+      <c r="D44">
+        <v>940</v>
+      </c>
+      <c r="E44">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>38</v>
+      </c>
+      <c r="B45" t="s">
+        <v>14</v>
+      </c>
+      <c r="C45">
+        <v>422</v>
+      </c>
+      <c r="D45">
+        <v>543</v>
+      </c>
+      <c r="E45">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>38</v>
+      </c>
+      <c r="B46" t="s">
+        <v>23</v>
+      </c>
+      <c r="C46">
+        <v>881</v>
+      </c>
+      <c r="D46">
+        <v>531</v>
+      </c>
+      <c r="E46">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B47" t="s">
+        <v>24</v>
+      </c>
+      <c r="C47">
+        <v>645</v>
+      </c>
+      <c r="D47">
+        <v>588</v>
+      </c>
+      <c r="E47">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>38</v>
+      </c>
+      <c r="B48" t="s">
+        <v>25</v>
+      </c>
+      <c r="C48">
+        <v>617</v>
+      </c>
+      <c r="D48">
+        <v>513</v>
+      </c>
+      <c r="E48">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>38</v>
+      </c>
+      <c r="B49" t="s">
+        <v>26</v>
+      </c>
+      <c r="C49">
+        <v>492</v>
+      </c>
+      <c r="D49">
+        <v>477</v>
+      </c>
+      <c r="E49">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B50" t="s">
+        <v>27</v>
+      </c>
+      <c r="C50">
+        <v>324</v>
+      </c>
+      <c r="D50">
+        <v>566</v>
+      </c>
+      <c r="E50">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51">
+        <v>300</v>
+      </c>
+      <c r="D51">
+        <v>616</v>
+      </c>
+      <c r="E51">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>38</v>
+      </c>
+      <c r="B52" t="s">
+        <v>29</v>
+      </c>
+      <c r="C52">
+        <v>297</v>
+      </c>
+      <c r="D52">
+        <v>606</v>
+      </c>
+      <c r="E52">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>38</v>
+      </c>
+      <c r="B53" t="s">
+        <v>30</v>
+      </c>
+      <c r="C53">
+        <v>396</v>
+      </c>
+      <c r="D53">
+        <v>609</v>
+      </c>
+      <c r="E53">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>38</v>
+      </c>
+      <c r="B54" t="s">
+        <v>12</v>
+      </c>
+      <c r="C54">
+        <v>600</v>
+      </c>
+      <c r="D54">
+        <v>563</v>
+      </c>
+      <c r="E54">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>38</v>
+      </c>
+      <c r="B55" t="s">
+        <v>31</v>
+      </c>
+      <c r="C55">
+        <v>745</v>
+      </c>
+      <c r="D55">
+        <v>539</v>
+      </c>
+      <c r="E55">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>38</v>
+      </c>
+      <c r="B56" t="s">
+        <v>32</v>
+      </c>
+      <c r="C56">
+        <v>787</v>
+      </c>
+      <c r="D56">
+        <v>490</v>
+      </c>
+      <c r="E56">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>38</v>
+      </c>
+      <c r="B57" t="s">
+        <v>33</v>
+      </c>
+      <c r="C57">
+        <v>818</v>
+      </c>
+      <c r="D57">
+        <v>680</v>
+      </c>
+      <c r="E57">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>38</v>
+      </c>
+      <c r="B58" t="s">
         <v>34</v>
       </c>
-      <c r="C3">
-        <v>1002</v>
-      </c>
-      <c r="D3">
-        <v>529</v>
-      </c>
-      <c r="E3">
-        <v>806</v>
+      <c r="C58">
+        <v>855</v>
+      </c>
+      <c r="D58">
+        <v>557</v>
+      </c>
+      <c r="E58">
+        <v>603</v>
       </c>
     </row>
   </sheetData>

</xml_diff>